<commit_message>
Expand audited five-school profiles to 296 and preserve uncertainty; fix narrow profile layout
</commit_message>
<xml_diff>
--- a/site/exports/hit-weihai-information.xlsx
+++ b/site/exports/hit-weihai-information.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="R3d50123b36a74270"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="经历" sheetId="2" r:id="Rd177e95c7d704597"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="导师" sheetId="3" r:id="Ra3009c4907fb4daa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="论文" sheetId="4" r:id="Rb794cf6bf8794fac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源" sheetId="5" r:id="R84856f2d539c4e27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="Rc73009707e724724"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="经历" sheetId="2" r:id="R65e2db4dd4184e55"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="导师" sheetId="3" r:id="Ra867646464184bad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="论文" sheetId="4" r:id="R0e84c6fecac54042"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源" sheetId="5" r:id="Rf6e5c5ecd2dc4784"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2498,7 +2498,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8bdc87732234007"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfca99cc3e8a844f9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19124,7 +19124,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R527b76a971d6460e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49f30e7845c34db0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19813,7 +19813,7 @@
         <x:v>active_officially_listed</x:v>
       </x:c>
       <x:c r="G19" s="6" t="str">
-        <x:v>本人页面列教授/博导，学校现任领导表列校长助理。专门实验室简介跳转认证，未绕过，个人主页导航待核。</x:v>
+        <x:v>本人页面列教授/博导，学校现任领导表列校长助理。专门实验室简介跳转认证，未绕过，个人主页导航待核。；任职已核实；专门个人简介跳转身份认证，未绕过；保留公开学校领导表的在职证据，暂不提供个人主页导航。</x:v>
       </x:c>
       <x:c r="H19" s="6" t="str"/>
       <x:c r="I19" s="6" t="str">
@@ -19832,7 +19832,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8fe1e1b2d6f84a67"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45e4e29eafb640b1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25582,7 +25582,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R251d89f53b014dfb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc2b4f673d164a27"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31330,7 +31330,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ea85a409c054e83"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d19966c8f3542e2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Expand verified breadth coverage to nine universities
</commit_message>
<xml_diff>
--- a/site/exports/hit-weihai-information.xlsx
+++ b/site/exports/hit-weihai-information.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="Rc73009707e724724"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="经历" sheetId="2" r:id="R65e2db4dd4184e55"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="导师" sheetId="3" r:id="Ra867646464184bad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="论文" sheetId="4" r:id="R0e84c6fecac54042"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源" sheetId="5" r:id="Rf6e5c5ecd2dc4784"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="R73e8205978394e6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="经历" sheetId="2" r:id="R490edfa934f34759"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="导师" sheetId="3" r:id="R639750f8b15042a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="论文" sheetId="4" r:id="R5de6022a1a264e26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源" sheetId="5" r:id="Rdb387c5af33e4fe7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -139,7 +139,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T5_0" displayName="T5_0" ref="A1:K62" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T7_0" displayName="T7_0" ref="A1:K62" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="姓名"/>
     <x:tableColumn id="2" name="校区"/>
@@ -158,7 +158,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="T5_1" displayName="T5_1" ref="A1:S367" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="T7_1" displayName="T7_1" ref="A1:S367" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="19">
     <x:tableColumn id="1" name="姓名"/>
     <x:tableColumn id="2" name="事件类型"/>
@@ -185,7 +185,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="T5_2" displayName="T5_2" ref="A1:L19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="T7_2" displayName="T7_2" ref="A1:L19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="姓名"/>
     <x:tableColumn id="2" name="导师姓名"/>
@@ -205,7 +205,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="T5_3" displayName="T5_3" ref="A1:L159" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="T7_3" displayName="T7_3" ref="A1:L159" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="姓名"/>
     <x:tableColumn id="2" name="标题"/>
@@ -225,7 +225,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="T5_4" displayName="T5_4" ref="A1:G249" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="T7_4" displayName="T7_4" ref="A1:G249" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="姓名"/>
     <x:tableColumn id="2" name="来源ID"/>
@@ -2498,7 +2498,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfca99cc3e8a844f9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb326d858b49f47a5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19124,7 +19124,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49f30e7845c34db0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f075c8624ed41a6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19832,7 +19832,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45e4e29eafb640b1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R122a2fe095064384"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19910,7 +19910,7 @@
         <x:v>https://doi.org/10.1016/j.jksuci.2024.102192</x:v>
       </x:c>
       <x:c r="F2" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G2" s="6" t="str">
         <x:v>https://repository.sutd.edu.sg/esploro/outputs/journalArticle/Enhanced-prediction-model-of-short-term-sea/9911686109846</x:v>
@@ -19919,7 +19919,7 @@
         <x:v>https://homepage.hit.edu.cn/jintao</x:v>
       </x:c>
       <x:c r="I2" s="6" t="str">
-        <x:v>previously_verified_institutional_metadata_preserved</x:v>
+        <x:v>保留此前独立机构元数据核验及原首篇书目，不称本轮重新读取。；previously_verified_institutional_metadata_preserved</x:v>
       </x:c>
       <x:c r="J2" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：保留此前独立机构元数据核验及原首篇书目，不称本轮重新读取。</x:v>
@@ -19946,7 +19946,7 @@
         <x:v>https://homepage.hit.edu.cn/jintao</x:v>
       </x:c>
       <x:c r="F3" s="6" t="str">
-        <x:v>conference_paper</x:v>
+        <x:v>会议论文；conference_paper</x:v>
       </x:c>
       <x:c r="G3" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/jintao</x:v>
@@ -19955,7 +19955,7 @@
         <x:v>https://homepage.hit.edu.cn/jintao</x:v>
       </x:c>
       <x:c r="I3" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J3" s="6" t="str">
         <x:v>题名Localiztion按官网原拼写保留，未修作出版商确证题名。 成果类型：会议论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -19982,7 +19982,7 @@
         <x:v>https://homepage.hit.edu.cn/jintao</x:v>
       </x:c>
       <x:c r="F4" s="6" t="str">
-        <x:v>conference_paper</x:v>
+        <x:v>会议论文；conference_paper</x:v>
       </x:c>
       <x:c r="G4" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/jintao</x:v>
@@ -19991,7 +19991,7 @@
         <x:v>https://homepage.hit.edu.cn/jintao</x:v>
       </x:c>
       <x:c r="I4" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J4" s="6" t="str">
         <x:v>成果类型：会议论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -20018,7 +20018,7 @@
         <x:v>https://homepage.hit.edu.cn/sunmingjian</x:v>
       </x:c>
       <x:c r="F5" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G5" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/sunmingjian</x:v>
@@ -20027,7 +20027,7 @@
         <x:v>https://homepage.hit.edu.cn/maly</x:v>
       </x:c>
       <x:c r="I5" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J5" s="6" t="str">
         <x:v>共同作者孙明健官方书目列Ma Liyong；本人当前主页仅有论文数量，未提供逐篇列表。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -20054,7 +20054,7 @@
         <x:v>https://homepage.hit.edu.cn/sunmingjian</x:v>
       </x:c>
       <x:c r="F6" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G6" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/sunmingjian</x:v>
@@ -20063,7 +20063,7 @@
         <x:v>https://homepage.hit.edu.cn/maly</x:v>
       </x:c>
       <x:c r="I6" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J6" s="6" t="str">
         <x:v>同院系共同作者官网明确列Liyong Ma；只保存元数据。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -20090,7 +20090,7 @@
         <x:v>https://homepage.hit.edu.cn/sunmingjian</x:v>
       </x:c>
       <x:c r="F7" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G7" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/sunmingjian</x:v>
@@ -20099,7 +20099,7 @@
         <x:v>https://homepage.hit.edu.cn/maly</x:v>
       </x:c>
       <x:c r="I7" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J7" s="6" t="str">
         <x:v>共同作者孙明健官网列Ma Liyong，团队成员栏明确中文姓名马立勇；不据共同作者推师承。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -20126,7 +20126,7 @@
         <x:v>https://homepage.hit.edu.cn/wangxiaoli</x:v>
       </x:c>
       <x:c r="F8" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G8" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/wangxiaoli</x:v>
@@ -20135,7 +20135,7 @@
         <x:v>https://homepage.hit.edu.cn/wangxiaoli</x:v>
       </x:c>
       <x:c r="I8" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J8" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -20162,7 +20162,7 @@
         <x:v>https://homepage.hit.edu.cn/wangxiaoli</x:v>
       </x:c>
       <x:c r="F9" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G9" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/wangxiaoli</x:v>
@@ -20171,7 +20171,7 @@
         <x:v>https://homepage.hit.edu.cn/wangxiaoli</x:v>
       </x:c>
       <x:c r="I9" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J9" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -20198,7 +20198,7 @@
         <x:v>https://www.jseepub.com/CN/article/downloadArticleFile.do?attachType=PDF&amp;id=5416</x:v>
       </x:c>
       <x:c r="F10" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G10" s="6" t="str">
         <x:v>https://www.jseepub.com/CN/article/downloadArticleFile.do?attachType=PDF&amp;id=5416</x:v>
@@ -20207,7 +20207,7 @@
         <x:v>https://homepage.hit.edu.cn/wangxiaoli</x:v>
       </x:c>
       <x:c r="I10" s="6" t="str">
-        <x:v>publisher_search_metadata_direct_pdf_unavailable</x:v>
+        <x:v>出版社搜索元数据，直接PDF不可用，不冒称PDF已读。；publisher_search_metadata_direct_pdf_unavailable</x:v>
       </x:c>
       <x:c r="J10" s="6" t="str">
         <x:v>出版社PDF题录及作者简介由检索索引读取，直接PDF获取失败；不称已验证可打开论文链接。 成果类型：期刊论文。 链接核验范围：出版社搜索元数据，直接PDF不可用，不冒称PDF已读。</x:v>
@@ -20234,7 +20234,7 @@
         <x:v>https://homepage.hit.edu.cn/sunmingjian</x:v>
       </x:c>
       <x:c r="F11" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G11" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/sunmingjian</x:v>
@@ -20243,7 +20243,7 @@
         <x:v>https://homepage.hit.edu.cn/sunmingjian</x:v>
       </x:c>
       <x:c r="I11" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J11" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -20270,7 +20270,7 @@
         <x:v>https://homepage.hit.edu.cn/sunmingjian</x:v>
       </x:c>
       <x:c r="F12" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G12" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/sunmingjian</x:v>
@@ -20279,7 +20279,7 @@
         <x:v>https://homepage.hit.edu.cn/sunmingjian</x:v>
       </x:c>
       <x:c r="I12" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J12" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -20306,7 +20306,7 @@
         <x:v>https://homepage.hit.edu.cn/sunmingjian</x:v>
       </x:c>
       <x:c r="F13" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G13" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/sunmingjian</x:v>
@@ -20315,7 +20315,7 @@
         <x:v>https://homepage.hit.edu.cn/sunmingjian</x:v>
       </x:c>
       <x:c r="I13" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J13" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -20342,7 +20342,7 @@
         <x:v>https://homepage.hit.edu.cn/denglibao</x:v>
       </x:c>
       <x:c r="F14" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G14" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/ueditor/jsp/upload/image/20240225/1708856001283036551.png</x:v>
@@ -20351,7 +20351,7 @@
         <x:v>https://homepage.hit.edu.cn/denglibao</x:v>
       </x:c>
       <x:c r="I14" s="6" t="str">
-        <x:v>official_embedded_publication_image_read</x:v>
+        <x:v>本人官网嵌入书目图片已读，不等于独立文章落地页或全文已读。；official_embedded_publication_image_read</x:v>
       </x:c>
       <x:c r="J14" s="6" t="str">
         <x:v>本人主页发表文章区嵌入图片第1条，人工视觉核读；未列页码/DOI。 成果类型：期刊论文。 链接核验范围：本人官网嵌入书目图片已读，不等于独立文章落地页或全文已读。</x:v>
@@ -20378,7 +20378,7 @@
         <x:v>https://homepage.hit.edu.cn/denglibao</x:v>
       </x:c>
       <x:c r="F15" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G15" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/ueditor/jsp/upload/image/20240225/1708856001283036551.png</x:v>
@@ -20387,7 +20387,7 @@
         <x:v>https://homepage.hit.edu.cn/denglibao</x:v>
       </x:c>
       <x:c r="I15" s="6" t="str">
-        <x:v>official_embedded_publication_image_read</x:v>
+        <x:v>本人官网嵌入书目图片已读，不等于独立文章落地页或全文已读。；official_embedded_publication_image_read</x:v>
       </x:c>
       <x:c r="J15" s="6" t="str">
         <x:v>本人主页书目图片第2条；不把图片URL当出版社单篇落地链接。 成果类型：期刊论文。 链接核验范围：本人官网嵌入书目图片已读，不等于独立文章落地页或全文已读。</x:v>
@@ -20414,7 +20414,7 @@
         <x:v>https://homepage.hit.edu.cn/denglibao</x:v>
       </x:c>
       <x:c r="F16" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G16" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/ueditor/jsp/upload/image/20240225/1708856001283036551.png</x:v>
@@ -20423,7 +20423,7 @@
         <x:v>https://homepage.hit.edu.cn/denglibao</x:v>
       </x:c>
       <x:c r="I16" s="6" t="str">
-        <x:v>official_embedded_publication_image_read</x:v>
+        <x:v>本人官网嵌入书目图片已读，不等于独立文章落地页或全文已读。；official_embedded_publication_image_read</x:v>
       </x:c>
       <x:c r="J16" s="6" t="str">
         <x:v>本人主页书目图片第3条仅列2023:1–22，未推定最终卷期。 成果类型：期刊论文。 链接核验范围：本人官网嵌入书目图片已读，不等于独立文章落地页或全文已读。</x:v>
@@ -20450,7 +20450,7 @@
         <x:v>https://homepage.hit.edu.cn/yangzhao</x:v>
       </x:c>
       <x:c r="F17" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G17" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/yangzhao</x:v>
@@ -20459,7 +20459,7 @@
         <x:v>https://homepage.hit.edu.cn/yangzhao</x:v>
       </x:c>
       <x:c r="I17" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J17" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -20486,7 +20486,7 @@
         <x:v>https://homepage.hit.edu.cn/yangzhao</x:v>
       </x:c>
       <x:c r="F18" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G18" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/yangzhao</x:v>
@@ -20495,7 +20495,7 @@
         <x:v>https://homepage.hit.edu.cn/yangzhao</x:v>
       </x:c>
       <x:c r="I18" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J18" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -20522,7 +20522,7 @@
         <x:v>https://homepage.hit.edu.cn/yangzhao</x:v>
       </x:c>
       <x:c r="F19" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G19" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/yangzhao</x:v>
@@ -20531,7 +20531,7 @@
         <x:v>https://homepage.hit.edu.cn/yangzhao</x:v>
       </x:c>
       <x:c r="I19" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J19" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -20558,7 +20558,7 @@
         <x:v>https://homepage.hit.edu.cn/luoqinghua</x:v>
       </x:c>
       <x:c r="F20" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G20" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/luoqinghua</x:v>
@@ -20567,7 +20567,7 @@
         <x:v>https://homepage.hit.edu.cn/luoqinghua</x:v>
       </x:c>
       <x:c r="I20" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J20" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -20594,7 +20594,7 @@
         <x:v>https://homepage.hit.edu.cn/luoqinghua</x:v>
       </x:c>
       <x:c r="F21" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G21" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/luoqinghua</x:v>
@@ -20603,7 +20603,7 @@
         <x:v>https://homepage.hit.edu.cn/luoqinghua</x:v>
       </x:c>
       <x:c r="I21" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J21" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -20630,7 +20630,7 @@
         <x:v>https://homepage.hit.edu.cn/luoqinghua</x:v>
       </x:c>
       <x:c r="F22" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G22" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/luoqinghua</x:v>
@@ -20639,7 +20639,7 @@
         <x:v>https://homepage.hit.edu.cn/luoqinghua</x:v>
       </x:c>
       <x:c r="I22" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J22" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -20668,7 +20668,7 @@
         <x:v>https://ietresearch.onlinelibrary.wiley.com/doi/10.1049/el.2019.1160</x:v>
       </x:c>
       <x:c r="F23" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G23" s="6" t="str">
         <x:v>https://ietresearch.onlinelibrary.wiley.com/doi/10.1049/el.2019.1160</x:v>
@@ -20677,7 +20677,7 @@
         <x:v>本人/同事官方论文列表与出版社同名HIT Weihai机构、雷达研究方向相符。</x:v>
       </x:c>
       <x:c r="I23" s="6" t="str">
-        <x:v>publisher_article_metadata_verified</x:v>
+        <x:v>出版社逐篇文章元数据及身份已核，不表示全文复制或完整论文库。；publisher_article_metadata_verified</x:v>
       </x:c>
       <x:c r="J23" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：出版社逐篇文章元数据及身份已核，不表示全文复制或完整论文库。</x:v>
@@ -20706,7 +20706,7 @@
         <x:v>https://iris.polito.it/retrieve/handle/11583/2999128/4416e6d0-8720-488b-8823-8cc0415838f4/Resource_Allocation_for_Multi-Satellite_Asynchronous_Transmission_in_Integrated_Communication_and_Navigation_Networks.pdf</x:v>
       </x:c>
       <x:c r="F24" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G24" s="6" t="str">
         <x:v>https://iris.polito.it/retrieve/handle/11583/2999128/4416e6d0-8720-488b-8823-8cc0415838f4/Resource_Allocation_for_Multi-Satellite_Asynchronous_Transmission_in_Integrated_Communication_and_Navigation_Networks.pdf</x:v>
@@ -20715,7 +20715,7 @@
         <x:v>https://homepage.hit.edu.cn/liugongliang</x:v>
       </x:c>
       <x:c r="I24" s="6" t="str">
-        <x:v>article_metadata_verified</x:v>
+        <x:v>逐篇书目元数据已核，不等于全文读取。；article_metadata_verified</x:v>
       </x:c>
       <x:c r="J24" s="6" t="str">
         <x:v>仅读取公开作者稿的书目及本人职业简历，不转载全文。 成果类型：期刊论文。 链接核验范围：逐篇书目元数据已核，不等于全文读取。</x:v>
@@ -20742,7 +20742,7 @@
         <x:v>https://homepage.hit.edu.cn/liugongliang</x:v>
       </x:c>
       <x:c r="F25" s="6" t="str">
-        <x:v>book</x:v>
+        <x:v>著作；book</x:v>
       </x:c>
       <x:c r="G25" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/liugongliang</x:v>
@@ -20751,7 +20751,7 @@
         <x:v>https://homepage.hit.edu.cn/liugongliang</x:v>
       </x:c>
       <x:c r="I25" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J25" s="6" t="str">
         <x:v>成果类型：著作。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -20780,7 +20780,7 @@
         <x:v>https://ietresearch.onlinelibrary.wiley.com/doi/10.1049/el.2019.1160</x:v>
       </x:c>
       <x:c r="F26" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G26" s="6" t="str">
         <x:v>https://ietresearch.onlinelibrary.wiley.com/doi/10.1049/el.2019.1160</x:v>
@@ -20789,7 +20789,7 @@
         <x:v>本人/同事官方论文列表与出版社同名HIT Weihai机构、雷达研究方向相符。</x:v>
       </x:c>
       <x:c r="I26" s="6" t="str">
-        <x:v>publisher_article_metadata_verified</x:v>
+        <x:v>出版社逐篇文章元数据及身份已核，不表示全文复制或完整论文库。；publisher_article_metadata_verified</x:v>
       </x:c>
       <x:c r="J26" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：出版社逐篇文章元数据及身份已核，不表示全文复制或完整论文库。</x:v>
@@ -20816,7 +20816,7 @@
         <x:v>https://homepage.hit.edu.cn/liuaijun</x:v>
       </x:c>
       <x:c r="F27" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G27" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/liuaijun</x:v>
@@ -20825,7 +20825,7 @@
         <x:v>https://homepage.hit.edu.cn/liuaijun</x:v>
       </x:c>
       <x:c r="I27" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J27" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -20852,7 +20852,7 @@
         <x:v>https://homepage.hit.edu.cn/liuaijun</x:v>
       </x:c>
       <x:c r="F28" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G28" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/liuaijun</x:v>
@@ -20861,7 +20861,7 @@
         <x:v>https://homepage.hit.edu.cn/liuaijun</x:v>
       </x:c>
       <x:c r="I28" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J28" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -20890,7 +20890,7 @@
         <x:v>https://doi.org/10.1109/MVT.2025.3586822</x:v>
       </x:c>
       <x:c r="F29" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G29" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/libo</x:v>
@@ -20899,7 +20899,7 @@
         <x:v>https://homepage.hit.edu.cn/libo</x:v>
       </x:c>
       <x:c r="I29" s="6" t="str">
-        <x:v>doi_explicitly_listed_on_official_profile</x:v>
+        <x:v>DOI由本人官网明确列示，独立文章页核验另行标记。；doi_explicitly_listed_on_official_profile</x:v>
       </x:c>
       <x:c r="J29" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：DOI由本人官网明确列示，独立文章页核验另行标记。</x:v>
@@ -20926,7 +20926,7 @@
         <x:v>https://homepage.hit.edu.cn/libo</x:v>
       </x:c>
       <x:c r="F30" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G30" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/libo</x:v>
@@ -20935,7 +20935,7 @@
         <x:v>https://homepage.hit.edu.cn/libo</x:v>
       </x:c>
       <x:c r="I30" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J30" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -20962,7 +20962,7 @@
         <x:v>https://homepage.hit.edu.cn/libo</x:v>
       </x:c>
       <x:c r="F31" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G31" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/libo</x:v>
@@ -20971,7 +20971,7 @@
         <x:v>https://homepage.hit.edu.cn/libo</x:v>
       </x:c>
       <x:c r="I31" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J31" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -20998,7 +20998,7 @@
         <x:v>https://homepage.hit.edu.cn/zhouzhiquan</x:v>
       </x:c>
       <x:c r="F32" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G32" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/zhouzhiquan</x:v>
@@ -21007,7 +21007,7 @@
         <x:v>https://homepage.hit.edu.cn/zhouzhiquan</x:v>
       </x:c>
       <x:c r="I32" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J32" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -21034,7 +21034,7 @@
         <x:v>https://homepage.hit.edu.cn/zhouzhiquan</x:v>
       </x:c>
       <x:c r="F33" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G33" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/zhouzhiquan</x:v>
@@ -21043,7 +21043,7 @@
         <x:v>https://homepage.hit.edu.cn/zhouzhiquan</x:v>
       </x:c>
       <x:c r="I33" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J33" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -21070,7 +21070,7 @@
         <x:v>https://homepage.hit.edu.cn/zhouzhiquan</x:v>
       </x:c>
       <x:c r="F34" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G34" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/zhouzhiquan</x:v>
@@ -21079,7 +21079,7 @@
         <x:v>https://homepage.hit.edu.cn/zhouzhiquan</x:v>
       </x:c>
       <x:c r="I34" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J34" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -21108,7 +21108,7 @@
         <x:v>https://www.jseepub.com/EN/10.23919/JSEE.2021.000005</x:v>
       </x:c>
       <x:c r="F35" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G35" s="6" t="str">
         <x:v>https://www.jseepub.com/EN/10.23919/JSEE.2021.000005</x:v>
@@ -21117,7 +21117,7 @@
         <x:v>https://homepage.hit.edu.cn/MingJin</x:v>
       </x:c>
       <x:c r="I35" s="6" t="str">
-        <x:v>publisher_article_page_verified</x:v>
+        <x:v>出版社逐篇元数据已核，不表示复制全文或完整成果库。；publisher_article_page_verified</x:v>
       </x:c>
       <x:c r="J35" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：出版社逐篇元数据已核，不表示复制全文或完整成果库。</x:v>
@@ -21144,7 +21144,7 @@
         <x:v>https://homepage.hit.edu.cn/yanfenggang</x:v>
       </x:c>
       <x:c r="F36" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G36" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/yanfenggang</x:v>
@@ -21153,7 +21153,7 @@
         <x:v>https://homepage.hit.edu.cn/MingJin</x:v>
       </x:c>
       <x:c r="I36" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J36" s="6" t="str">
         <x:v>本人主页未列逐篇成果；同院共同作者闫锋刚官方书目及出版社同人简历交叉确认作者，不据此推师承。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -21180,7 +21180,7 @@
         <x:v>https://homepage.hit.edu.cn/LiuS</x:v>
       </x:c>
       <x:c r="F37" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G37" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/LiuS</x:v>
@@ -21189,7 +21189,7 @@
         <x:v>https://homepage.hit.edu.cn/MingJin</x:v>
       </x:c>
       <x:c r="I37" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J37" s="6" t="str">
         <x:v>取共同作者刘帅官网中文列表已出版条目；未把英文旧栏accepted状态覆盖中文卷页。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -21218,7 +21218,7 @@
         <x:v>https://www.jseepub.com/EN/10.23919/JSEE.2021.000005</x:v>
       </x:c>
       <x:c r="F38" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G38" s="6" t="str">
         <x:v>https://www.jseepub.com/EN/10.23919/JSEE.2021.000005</x:v>
@@ -21227,7 +21227,7 @@
         <x:v>https://homepage.hit.edu.cn/LiuS</x:v>
       </x:c>
       <x:c r="I38" s="6" t="str">
-        <x:v>publisher_article_page_verified</x:v>
+        <x:v>出版社逐篇元数据已核，不表示复制全文或完整成果库。；publisher_article_page_verified</x:v>
       </x:c>
       <x:c r="J38" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：出版社逐篇元数据已核，不表示复制全文或完整成果库。</x:v>
@@ -21254,7 +21254,7 @@
         <x:v>https://homepage.hit.edu.cn/LiuS</x:v>
       </x:c>
       <x:c r="F39" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G39" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/LiuS</x:v>
@@ -21263,7 +21263,7 @@
         <x:v>https://homepage.hit.edu.cn/LiuS</x:v>
       </x:c>
       <x:c r="I39" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J39" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -21290,7 +21290,7 @@
         <x:v>https://homepage.hit.edu.cn/LiuS</x:v>
       </x:c>
       <x:c r="F40" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G40" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/LiuS</x:v>
@@ -21299,7 +21299,7 @@
         <x:v>https://homepage.hit.edu.cn/LiuS</x:v>
       </x:c>
       <x:c r="I40" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J40" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -21326,7 +21326,7 @@
         <x:v>https://homepage.hit.edu.cn/yanfenggang</x:v>
       </x:c>
       <x:c r="F41" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G41" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/yanfenggang</x:v>
@@ -21335,7 +21335,7 @@
         <x:v>https://homepage.hit.edu.cn/yanfenggang</x:v>
       </x:c>
       <x:c r="I41" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J41" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -21362,7 +21362,7 @@
         <x:v>https://homepage.hit.edu.cn/yanfenggang</x:v>
       </x:c>
       <x:c r="F42" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G42" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/yanfenggang</x:v>
@@ -21371,7 +21371,7 @@
         <x:v>https://homepage.hit.edu.cn/yanfenggang</x:v>
       </x:c>
       <x:c r="I42" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J42" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -21400,7 +21400,7 @@
         <x:v>https://www.jseepub.com/EN/10.23919/JSEE.2021.000005</x:v>
       </x:c>
       <x:c r="F43" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G43" s="6" t="str">
         <x:v>https://www.jseepub.com/EN/10.23919/JSEE.2021.000005</x:v>
@@ -21409,7 +21409,7 @@
         <x:v>https://homepage.hit.edu.cn/yanfenggang</x:v>
       </x:c>
       <x:c r="I43" s="6" t="str">
-        <x:v>publisher_article_page_verified</x:v>
+        <x:v>出版社逐篇元数据已核，不表示复制全文或完整成果库。；publisher_article_page_verified</x:v>
       </x:c>
       <x:c r="J43" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：出版社逐篇元数据已核，不表示复制全文或完整成果库。</x:v>
@@ -21436,7 +21436,7 @@
         <x:v>https://homepage.hit.edu.cn/zhouzhiquan</x:v>
       </x:c>
       <x:c r="F44" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G44" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/zhouzhiquan</x:v>
@@ -21445,7 +21445,7 @@
         <x:v>https://homepage.hit.edu.cn/zhaozhanfeng</x:v>
       </x:c>
       <x:c r="I44" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J44" s="6" t="str">
         <x:v>本人论文区空；共同作者周志权官方书目列作者，且团队成员明确中文赵占锋及相同质谱仪方向。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -21472,7 +21472,7 @@
         <x:v>https://homepage.hit.edu.cn/zhouzhiquan</x:v>
       </x:c>
       <x:c r="F45" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G45" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/zhouzhiquan</x:v>
@@ -21481,7 +21481,7 @@
         <x:v>https://homepage.hit.edu.cn/zhaozhanfeng</x:v>
       </x:c>
       <x:c r="I45" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J45" s="6" t="str">
         <x:v>来自共同作者周志权官网，只收元数据，不据共同作者推导师。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -21508,7 +21508,7 @@
         <x:v>https://homepage.hit.edu.cn/zhouzhiquan</x:v>
       </x:c>
       <x:c r="F46" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G46" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/zhouzhiquan</x:v>
@@ -21517,7 +21517,7 @@
         <x:v>https://homepage.hit.edu.cn/zhaozhanfeng</x:v>
       </x:c>
       <x:c r="I46" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J46" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -21544,7 +21544,7 @@
         <x:v>https://homepage.hit.edu.cn/qixiaohui</x:v>
       </x:c>
       <x:c r="F47" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G47" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/qixiaohui</x:v>
@@ -21553,7 +21553,7 @@
         <x:v>https://homepage.hit.edu.cn/qixiaohui</x:v>
       </x:c>
       <x:c r="I47" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J47" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -21580,7 +21580,7 @@
         <x:v>https://homepage.hit.edu.cn/qixiaohui</x:v>
       </x:c>
       <x:c r="F48" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G48" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/qixiaohui</x:v>
@@ -21589,7 +21589,7 @@
         <x:v>https://homepage.hit.edu.cn/qixiaohui</x:v>
       </x:c>
       <x:c r="I48" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J48" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -21616,7 +21616,7 @@
         <x:v>https://homepage.hit.edu.cn/qixiaohui</x:v>
       </x:c>
       <x:c r="F49" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G49" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/qixiaohui</x:v>
@@ -21625,7 +21625,7 @@
         <x:v>https://homepage.hit.edu.cn/qixiaohui</x:v>
       </x:c>
       <x:c r="I49" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J49" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -21652,7 +21652,7 @@
         <x:v>https://homepage.hit.edu.cn/WeiZheng</x:v>
       </x:c>
       <x:c r="F50" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G50" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/WeiZheng</x:v>
@@ -21661,7 +21661,7 @@
         <x:v>https://homepage.hit.edu.cn/WeiZheng</x:v>
       </x:c>
       <x:c r="I50" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J50" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -21688,7 +21688,7 @@
         <x:v>https://homepage.hit.edu.cn/WeiZheng</x:v>
       </x:c>
       <x:c r="F51" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G51" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/WeiZheng</x:v>
@@ -21697,7 +21697,7 @@
         <x:v>https://homepage.hit.edu.cn/WeiZheng</x:v>
       </x:c>
       <x:c r="I51" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J51" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -21724,7 +21724,7 @@
         <x:v>https://homepage.hit.edu.cn/WeiZheng</x:v>
       </x:c>
       <x:c r="F52" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G52" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/WeiZheng</x:v>
@@ -21733,7 +21733,7 @@
         <x:v>https://homepage.hit.edu.cn/WeiZheng</x:v>
       </x:c>
       <x:c r="I52" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J52" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -21760,7 +21760,7 @@
         <x:v>https://homepage.hit.edu.cn/whwangjun</x:v>
       </x:c>
       <x:c r="F53" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G53" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/whwangjun</x:v>
@@ -21769,7 +21769,7 @@
         <x:v>https://homepage.hit.edu.cn/whwangjun</x:v>
       </x:c>
       <x:c r="I53" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J53" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -21796,7 +21796,7 @@
         <x:v>https://homepage.hit.edu.cn/whwangjun</x:v>
       </x:c>
       <x:c r="F54" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G54" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/whwangjun</x:v>
@@ -21805,7 +21805,7 @@
         <x:v>https://homepage.hit.edu.cn/whwangjun</x:v>
       </x:c>
       <x:c r="I54" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J54" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -21832,7 +21832,7 @@
         <x:v>https://homepage.hit.edu.cn/whwangjun</x:v>
       </x:c>
       <x:c r="F55" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G55" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/whwangjun</x:v>
@@ -21841,7 +21841,7 @@
         <x:v>https://homepage.hit.edu.cn/whwangjun</x:v>
       </x:c>
       <x:c r="I55" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J55" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -21868,7 +21868,7 @@
         <x:v>https://homepage.hit.edu.cn/xinmingrui</x:v>
       </x:c>
       <x:c r="F56" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G56" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/xinmingrui</x:v>
@@ -21877,7 +21877,7 @@
         <x:v>https://homepage.hit.edu.cn/xinmingrui</x:v>
       </x:c>
       <x:c r="I56" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J56" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -21904,7 +21904,7 @@
         <x:v>https://homepage.hit.edu.cn/xinmingrui</x:v>
       </x:c>
       <x:c r="F57" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G57" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/xinmingrui</x:v>
@@ -21913,7 +21913,7 @@
         <x:v>https://homepage.hit.edu.cn/xinmingrui</x:v>
       </x:c>
       <x:c r="I57" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J57" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -21940,7 +21940,7 @@
         <x:v>https://www.mdpi.com/2072-4292/17/2/295</x:v>
       </x:c>
       <x:c r="F58" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G58" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/wangchenxu</x:v>
@@ -21949,7 +21949,7 @@
         <x:v>https://homepage.hit.edu.cn/wangchenxu</x:v>
       </x:c>
       <x:c r="I58" s="6" t="str">
-        <x:v>publisher_index_title_match_landing_429_unverified</x:v>
+        <x:v>出版社检索索引题名匹配，落地页429未核、未重试；不声称直接逐页读到。；publisher_index_title_match_landing_429_unverified</x:v>
       </x:c>
       <x:c r="J58" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：出版社检索索引题名匹配，落地页429未核、未重试；不声称直接逐页读到。</x:v>
@@ -21976,7 +21976,7 @@
         <x:v>https://homepage.hit.edu.cn/wangchenxu</x:v>
       </x:c>
       <x:c r="F59" s="6" t="str">
-        <x:v>conference_paper</x:v>
+        <x:v>会议论文；conference_paper</x:v>
       </x:c>
       <x:c r="G59" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/wangchenxu</x:v>
@@ -21985,7 +21985,7 @@
         <x:v>https://homepage.hit.edu.cn/wangchenxu</x:v>
       </x:c>
       <x:c r="I59" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J59" s="6" t="str">
         <x:v>成果类型：会议论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -22012,7 +22012,7 @@
         <x:v>https://www.mdpi.com/2077-1312/11/7/1352</x:v>
       </x:c>
       <x:c r="F60" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G60" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/wangchenxu</x:v>
@@ -22021,7 +22021,7 @@
         <x:v>https://homepage.hit.edu.cn/wangchenxu</x:v>
       </x:c>
       <x:c r="I60" s="6" t="str">
-        <x:v>publisher_index_title_match_landing_429_unverified</x:v>
+        <x:v>出版社检索索引题名匹配，落地页429未核、未重试；不声称直接逐页读到。；publisher_index_title_match_landing_429_unverified</x:v>
       </x:c>
       <x:c r="J60" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：出版社检索索引题名匹配，落地页429未核、未重试；不声称直接逐页读到。</x:v>
@@ -22048,7 +22048,7 @@
         <x:v>https://homepage.hit.edu.cn/wangxinsheng</x:v>
       </x:c>
       <x:c r="F61" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G61" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/wangxinsheng</x:v>
@@ -22057,7 +22057,7 @@
         <x:v>https://homepage.hit.edu.cn/wangxinsheng</x:v>
       </x:c>
       <x:c r="I61" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J61" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -22084,7 +22084,7 @@
         <x:v>https://homepage.hit.edu.cn/wangxinsheng</x:v>
       </x:c>
       <x:c r="F62" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G62" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/wangxinsheng</x:v>
@@ -22093,7 +22093,7 @@
         <x:v>https://homepage.hit.edu.cn/wangxinsheng</x:v>
       </x:c>
       <x:c r="I62" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J62" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -22120,7 +22120,7 @@
         <x:v>https://homepage.hit.edu.cn/wangxinsheng</x:v>
       </x:c>
       <x:c r="F63" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G63" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/wangxinsheng</x:v>
@@ -22129,7 +22129,7 @@
         <x:v>https://homepage.hit.edu.cn/wangxinsheng</x:v>
       </x:c>
       <x:c r="I63" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J63" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -22156,7 +22156,7 @@
         <x:v>https://aces-society.org/includes/downloadpaper.php?nf=18-11-4&amp;of=ACES_Journal_November_2018_Paper_4</x:v>
       </x:c>
       <x:c r="F64" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G64" s="6" t="str">
         <x:v>https://aces-society.org/includes/downloadpaper.php?nf=18-11-4&amp;of=ACES_Journal_November_2018_Paper_4</x:v>
@@ -22165,7 +22165,7 @@
         <x:v>出版社作者机构HIT Weihai、学位年份与本人官网匹配</x:v>
       </x:c>
       <x:c r="I64" s="6" t="str">
-        <x:v>publisher_pdf_metadata_verified</x:v>
+        <x:v>正式出版社PDF书目或作者简介已核；只保留结构化事实，不发布全文。；publisher_pdf_metadata_verified</x:v>
       </x:c>
       <x:c r="J64" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：正式出版社PDF书目或作者简介已核；只保留结构化事实，不发布全文。</x:v>
@@ -22190,7 +22190,7 @@
         <x:v>https://homepage.hit.edu.cn/songlizhong</x:v>
       </x:c>
       <x:c r="F65" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G65" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/songlizhong</x:v>
@@ -22199,7 +22199,7 @@
         <x:v>https://homepage.hit.edu.cn/songlizhong</x:v>
       </x:c>
       <x:c r="I65" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J65" s="6" t="str">
         <x:v>官网发表时间空白，只列卷期；未凭卷号倒推出版年。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -22224,7 +22224,7 @@
         <x:v>https://homepage.hit.edu.cn/songlizhong</x:v>
       </x:c>
       <x:c r="F66" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G66" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/songlizhong</x:v>
@@ -22233,7 +22233,7 @@
         <x:v>https://homepage.hit.edu.cn/songlizhong</x:v>
       </x:c>
       <x:c r="I66" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J66" s="6" t="str">
         <x:v>官网发表时间空白，只列卷期；未凭卷号倒推出版年。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -22258,7 +22258,7 @@
         <x:v>https://homepage.hit.edu.cn/maxiujuan</x:v>
       </x:c>
       <x:c r="F67" s="6" t="str">
-        <x:v>book</x:v>
+        <x:v>著作；book</x:v>
       </x:c>
       <x:c r="G67" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/maxiujuan</x:v>
@@ -22267,7 +22267,7 @@
         <x:v>https://homepage.hit.edu.cn/maxiujuan</x:v>
       </x:c>
       <x:c r="I67" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J67" s="6" t="str">
         <x:v>官网列教材题名与编写参与，未给版本、出版年及出版社；不从其他同名教材猜填。 成果类型：著作。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -22292,7 +22292,7 @@
         <x:v>https://homepage.hit.edu.cn/maxiujuan</x:v>
       </x:c>
       <x:c r="F68" s="6" t="str">
-        <x:v>book</x:v>
+        <x:v>著作；book</x:v>
       </x:c>
       <x:c r="G68" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/maxiujuan</x:v>
@@ -22301,7 +22301,7 @@
         <x:v>https://homepage.hit.edu.cn/maxiujuan</x:v>
       </x:c>
       <x:c r="I68" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J68" s="6" t="str">
         <x:v>官网列教材题名与编写参与，未给版本、出版年及出版社；不从其他同名教材猜填。 成果类型：著作。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -22326,7 +22326,7 @@
         <x:v>https://homepage.hit.edu.cn/maxiujuan</x:v>
       </x:c>
       <x:c r="F69" s="6" t="str">
-        <x:v>book</x:v>
+        <x:v>著作；book</x:v>
       </x:c>
       <x:c r="G69" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/maxiujuan</x:v>
@@ -22335,7 +22335,7 @@
         <x:v>https://homepage.hit.edu.cn/maxiujuan</x:v>
       </x:c>
       <x:c r="I69" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J69" s="6" t="str">
         <x:v>官网列教材题名与编写参与，未给版本、出版年及出版社；不从其他同名教材猜填。 成果类型：著作。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -22364,7 +22364,7 @@
         <x:v>https://xuebao.neu.edu.cn/natural/CN/abstract/abstract5207.shtml</x:v>
       </x:c>
       <x:c r="F70" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G70" s="6" t="str">
         <x:v>https://xuebao.neu.edu.cn/natural/CN/abstract/abstract5207.shtml</x:v>
@@ -22373,7 +22373,7 @@
         <x:v>https://xuebao.neu.edu.cn/natural/CN/abstract/abstract5207.shtml</x:v>
       </x:c>
       <x:c r="I70" s="6" t="str">
-        <x:v>publisher_article_page_verified</x:v>
+        <x:v>出版社逐篇元数据已核，不表示复制全文或完整成果库。；publisher_article_page_verified</x:v>
       </x:c>
       <x:c r="J70" s="6" t="str">
         <x:v>作者中文姓名、威海院系及机器人研究方向一致；合著关系不作为导师关系证据。 成果类型：期刊论文。 链接核验范围：出版社逐篇元数据已核，不表示复制全文或完整成果库。</x:v>
@@ -22400,7 +22400,7 @@
         <x:v>https://homepage.hit.edu.cn/huanghaibin</x:v>
       </x:c>
       <x:c r="F71" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G71" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/huanghaibin</x:v>
@@ -22409,7 +22409,7 @@
         <x:v>https://homepage.hit.edu.cn/huanghaibin</x:v>
       </x:c>
       <x:c r="I71" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J71" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -22436,7 +22436,7 @@
         <x:v>https://homepage.hit.edu.cn/huanghaibin</x:v>
       </x:c>
       <x:c r="F72" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G72" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/huanghaibin</x:v>
@@ -22445,7 +22445,7 @@
         <x:v>https://homepage.hit.edu.cn/huanghaibin</x:v>
       </x:c>
       <x:c r="I72" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J72" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -22472,7 +22472,7 @@
         <x:v>https://homepage.hit.edu.cn/huanghaibin</x:v>
       </x:c>
       <x:c r="F73" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G73" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/huanghaibin</x:v>
@@ -22481,7 +22481,7 @@
         <x:v>https://homepage.hit.edu.cn/huanghaibin</x:v>
       </x:c>
       <x:c r="I73" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J73" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -22508,7 +22508,7 @@
         <x:v>https://homepage.hit.edu.cn/zhangjingyu</x:v>
       </x:c>
       <x:c r="F74" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G74" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/zhangjingyu</x:v>
@@ -22517,7 +22517,7 @@
         <x:v>https://homepage.hit.edu.cn/zhangjingyu</x:v>
       </x:c>
       <x:c r="I74" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J74" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -22544,7 +22544,7 @@
         <x:v>https://homepage.hit.edu.cn/zhangjingyu</x:v>
       </x:c>
       <x:c r="F75" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G75" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/zhangjingyu</x:v>
@@ -22553,7 +22553,7 @@
         <x:v>https://homepage.hit.edu.cn/zhangjingyu</x:v>
       </x:c>
       <x:c r="I75" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J75" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -22580,7 +22580,7 @@
         <x:v>https://homepage.hit.edu.cn/zhangjingyu</x:v>
       </x:c>
       <x:c r="F76" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G76" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/zhangjingyu</x:v>
@@ -22589,7 +22589,7 @@
         <x:v>https://homepage.hit.edu.cn/zhangjingyu</x:v>
       </x:c>
       <x:c r="I76" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J76" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -22616,7 +22616,7 @@
         <x:v>https://homepage.hit.edu.cn/zhuangyufei</x:v>
       </x:c>
       <x:c r="F77" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G77" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/zhuangyufei</x:v>
@@ -22625,7 +22625,7 @@
         <x:v>https://homepage.hit.edu.cn/zhuangyufei</x:v>
       </x:c>
       <x:c r="I77" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J77" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -22652,7 +22652,7 @@
         <x:v>https://homepage.hit.edu.cn/zhuangyufei</x:v>
       </x:c>
       <x:c r="F78" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G78" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/zhuangyufei</x:v>
@@ -22661,7 +22661,7 @@
         <x:v>https://homepage.hit.edu.cn/zhuangyufei</x:v>
       </x:c>
       <x:c r="I78" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J78" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -22688,7 +22688,7 @@
         <x:v>https://homepage.hit.edu.cn/zhuangyufei</x:v>
       </x:c>
       <x:c r="F79" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G79" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/zhuangyufei</x:v>
@@ -22697,7 +22697,7 @@
         <x:v>https://homepage.hit.edu.cn/zhuangyufei</x:v>
       </x:c>
       <x:c r="I79" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J79" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -22724,7 +22724,7 @@
         <x:v>https://homepage.hit.edu.cn/renxiuyun</x:v>
       </x:c>
       <x:c r="F80" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G80" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/renxiuyun</x:v>
@@ -22733,7 +22733,7 @@
         <x:v>https://homepage.hit.edu.cn/renxiuyun</x:v>
       </x:c>
       <x:c r="I80" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J80" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -22760,7 +22760,7 @@
         <x:v>https://homepage.hit.edu.cn/renxiuyun</x:v>
       </x:c>
       <x:c r="F81" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G81" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/renxiuyun</x:v>
@@ -22769,7 +22769,7 @@
         <x:v>https://homepage.hit.edu.cn/renxiuyun</x:v>
       </x:c>
       <x:c r="I81" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J81" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -22796,7 +22796,7 @@
         <x:v>https://homepage.hit.edu.cn/renxiuyun</x:v>
       </x:c>
       <x:c r="F82" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G82" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/renxiuyun</x:v>
@@ -22805,7 +22805,7 @@
         <x:v>https://homepage.hit.edu.cn/renxiuyun</x:v>
       </x:c>
       <x:c r="I82" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J82" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -22834,7 +22834,7 @@
         <x:v>https://doi.org/10.1109/JIOT.2025.3526154</x:v>
       </x:c>
       <x:c r="F83" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G83" s="6" t="str">
         <x:v>https://iris.polito.it/retrieve/handle/11583/2999128/4416e6d0-8720-488b-8823-8cc0415838f4/Resource_Allocation_for_Multi-Satellite_Asynchronous_Transmission_in_Integrated_Communication_and_Navigation_Networks.pdf</x:v>
@@ -22843,7 +22843,7 @@
         <x:v>https://homepage.hit.edu.cn/kangwenjing</x:v>
       </x:c>
       <x:c r="I83" s="6" t="str">
-        <x:v>article_metadata_verified</x:v>
+        <x:v>文章书目元数据已核；不等于全部成果或全文发布。；article_metadata_verified</x:v>
       </x:c>
       <x:c r="J83" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：文章书目元数据已核；不等于全部成果或全文发布。</x:v>
@@ -22870,7 +22870,7 @@
         <x:v>https://homepage.hit.edu.cn/meiyingjie</x:v>
       </x:c>
       <x:c r="F84" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G84" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/meiyingjie</x:v>
@@ -22879,7 +22879,7 @@
         <x:v>https://homepage.hit.edu.cn/meiyingjie</x:v>
       </x:c>
       <x:c r="I84" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J84" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -22906,7 +22906,7 @@
         <x:v>https://homepage.hit.edu.cn/meiyingjie</x:v>
       </x:c>
       <x:c r="F85" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G85" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/meiyingjie</x:v>
@@ -22915,7 +22915,7 @@
         <x:v>https://homepage.hit.edu.cn/meiyingjie</x:v>
       </x:c>
       <x:c r="I85" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J85" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -22942,7 +22942,7 @@
         <x:v>https://homepage.hit.edu.cn/meiyingjie</x:v>
       </x:c>
       <x:c r="F86" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G86" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/meiyingjie</x:v>
@@ -22951,7 +22951,7 @@
         <x:v>https://homepage.hit.edu.cn/meiyingjie</x:v>
       </x:c>
       <x:c r="I86" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J86" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -22980,7 +22980,7 @@
         <x:v>https://www.nature.com/articles/s41467-024-49569-3</x:v>
       </x:c>
       <x:c r="F87" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G87" s="6" t="str">
         <x:v>https://www.nature.com/articles/s41467-024-49569-3</x:v>
@@ -22989,7 +22989,7 @@
         <x:v>https://www.nature.com/articles/s41467-024-49569-3</x:v>
       </x:c>
       <x:c r="I87" s="6" t="str">
-        <x:v>publisher_article_page_verified</x:v>
+        <x:v>出版社逐篇元数据已核，不表示复制全文或完整成果库。；publisher_article_page_verified</x:v>
       </x:c>
       <x:c r="J87" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：出版社逐篇元数据已核，不表示复制全文或完整成果库。</x:v>
@@ -23016,7 +23016,7 @@
         <x:v>https://homepage.hit.edu.cn/sunfenghao</x:v>
       </x:c>
       <x:c r="F88" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G88" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/sunfenghao</x:v>
@@ -23025,7 +23025,7 @@
         <x:v>https://homepage.hit.edu.cn/sunfenghao</x:v>
       </x:c>
       <x:c r="I88" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J88" s="6" t="str">
         <x:v>题名和作者缩写按本人主页保留；未逐篇出版商核验，官网题名ionizations与吴健主页ionization存在单复数差异。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -23052,7 +23052,7 @@
         <x:v>https://homepage.hit.edu.cn/sunfenghao</x:v>
       </x:c>
       <x:c r="F89" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G89" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/sunfenghao</x:v>
@@ -23061,7 +23061,7 @@
         <x:v>https://homepage.hit.edu.cn/sunfenghao</x:v>
       </x:c>
       <x:c r="I89" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J89" s="6" t="str">
         <x:v>作者缩写及两名H. Li按本人主页原样保留，不自行合并同缩写作者。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -23090,7 +23090,7 @@
         <x:v>https://www.spacejournal.cn/hwyjggc/article/doi/10.3788/IRLA20240373</x:v>
       </x:c>
       <x:c r="F90" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G90" s="6" t="str">
         <x:v>https://www.spacejournal.cn/hwyjggc/article/doi/10.3788/IRLA20240373</x:v>
@@ -23099,7 +23099,7 @@
         <x:v>https://www.spacejournal.cn/hwyjggc/article/doi/10.3788/IRLA20240373</x:v>
       </x:c>
       <x:c r="I90" s="6" t="str">
-        <x:v>publisher_metadata_indexed_page_not_verified</x:v>
+        <x:v>仅期刊官方索引书目已核，文章原页未直接核实。；publisher_metadata_indexed_page_not_verified</x:v>
       </x:c>
       <x:c r="J90" s="6" t="str">
         <x:v>仅以期刊公开索引书目为据，直读返回420。文章号采用页面引用格式20240373，而非导航截断的202403。作者单位及研究方向与本人一致。 成果类型：期刊论文。 链接核验范围：仅期刊官方索引书目已核，文章原页未直接核实。</x:v>
@@ -23126,7 +23126,7 @@
         <x:v>https://homepage.hit.edu.cn/liuzhiyong</x:v>
       </x:c>
       <x:c r="F91" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G91" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/liuzhiyong</x:v>
@@ -23135,7 +23135,7 @@
         <x:v>https://homepage.hit.edu.cn/liuzhiyong</x:v>
       </x:c>
       <x:c r="I91" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J91" s="6" t="str">
         <x:v>本人官网英文Selected Publications列2026，卷页和DOI未披露；不是独立出版核验。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -23162,7 +23162,7 @@
         <x:v>https://homepage.hit.edu.cn/liuzhiyong</x:v>
       </x:c>
       <x:c r="F92" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G92" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/liuzhiyong</x:v>
@@ -23171,7 +23171,7 @@
         <x:v>https://homepage.hit.edu.cn/liuzhiyong</x:v>
       </x:c>
       <x:c r="I92" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J92" s="6" t="str">
         <x:v>年份及作者顺序按本人官网英文Selected Publications。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -23198,7 +23198,7 @@
         <x:v>https://homepage.hit.edu.cn/liuzhiyong</x:v>
       </x:c>
       <x:c r="F93" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G93" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/liuzhiyong</x:v>
@@ -23207,7 +23207,7 @@
         <x:v>https://homepage.hit.edu.cn/liuzhiyong</x:v>
       </x:c>
       <x:c r="I93" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J93" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -23234,7 +23234,7 @@
         <x:v>https://homepage.hit.edu.cn/jiangxu</x:v>
       </x:c>
       <x:c r="F94" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G94" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/jiangxu</x:v>
@@ -23243,7 +23243,7 @@
         <x:v>https://homepage.hit.edu.cn/jiangxu</x:v>
       </x:c>
       <x:c r="I94" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J94" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -23270,7 +23270,7 @@
         <x:v>https://homepage.hit.edu.cn/jiangxu</x:v>
       </x:c>
       <x:c r="F95" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G95" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/jiangxu</x:v>
@@ -23279,7 +23279,7 @@
         <x:v>https://homepage.hit.edu.cn/jiangxu</x:v>
       </x:c>
       <x:c r="I95" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J95" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -23306,7 +23306,7 @@
         <x:v>https://homepage.hit.edu.cn/jiangxu</x:v>
       </x:c>
       <x:c r="F96" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G96" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/jiangxu</x:v>
@@ -23315,7 +23315,7 @@
         <x:v>https://homepage.hit.edu.cn/jiangxu</x:v>
       </x:c>
       <x:c r="I96" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J96" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -23344,7 +23344,7 @@
         <x:v>https://www.jas.shu.edu.cn/CN/abstract/abstract1263.shtml</x:v>
       </x:c>
       <x:c r="F97" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G97" s="6" t="str">
         <x:v>https://www.jas.shu.edu.cn/CN/abstract/abstract1263.shtml</x:v>
@@ -23353,7 +23353,7 @@
         <x:v>https://www.jas.shu.edu.cn/CN/abstract/abstract1263.shtml</x:v>
       </x:c>
       <x:c r="I97" s="6" t="str">
-        <x:v>publisher_article_page_verified</x:v>
+        <x:v>出版社逐篇元数据已核，不表示复制全文或完整成果库。；publisher_article_page_verified</x:v>
       </x:c>
       <x:c r="J97" s="6" t="str">
         <x:v>同校通信学科及本人教育时间匹配；不以王钢、李博等合著关系推定师承。 成果类型：期刊论文。 链接核验范围：出版社逐篇元数据已核，不表示复制全文或完整成果库。</x:v>
@@ -23382,7 +23382,7 @@
         <x:v>https://doi.org/10.1109/JIOT.2025.3526154</x:v>
       </x:c>
       <x:c r="F98" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G98" s="6" t="str">
         <x:v>https://iris.polito.it/retrieve/handle/11583/2999128/4416e6d0-8720-488b-8823-8cc0415838f4/Resource_Allocation_for_Multi-Satellite_Asynchronous_Transmission_in_Integrated_Communication_and_Navigation_Networks.pdf</x:v>
@@ -23391,7 +23391,7 @@
         <x:v>https://homepage.hit.edu.cn/maruofeihit</x:v>
       </x:c>
       <x:c r="I98" s="6" t="str">
-        <x:v>article_metadata_verified</x:v>
+        <x:v>文章书目元数据已核；不等于全部成果或全文发布。；article_metadata_verified</x:v>
       </x:c>
       <x:c r="J98" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：文章书目元数据已核；不等于全部成果或全文发布。</x:v>
@@ -23418,7 +23418,7 @@
         <x:v>https://homepage.hit.edu.cn/maruofeihit</x:v>
       </x:c>
       <x:c r="F99" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G99" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/maruofeihit</x:v>
@@ -23427,7 +23427,7 @@
         <x:v>https://homepage.hit.edu.cn/maruofeihit</x:v>
       </x:c>
       <x:c r="I99" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J99" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -23454,7 +23454,7 @@
         <x:v>https://homepage.hit.edu.cn/maruofeihit</x:v>
       </x:c>
       <x:c r="F100" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G100" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/maruofeihit</x:v>
@@ -23463,7 +23463,7 @@
         <x:v>https://homepage.hit.edu.cn/maruofeihit</x:v>
       </x:c>
       <x:c r="I100" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J100" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -23490,7 +23490,7 @@
         <x:v>https://homepage.hit.edu.cn/wangxiuhong</x:v>
       </x:c>
       <x:c r="F101" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G101" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/wangxiuhong</x:v>
@@ -23499,7 +23499,7 @@
         <x:v>https://homepage.hit.edu.cn/wangxiuhong</x:v>
       </x:c>
       <x:c r="I101" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J101" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -23526,7 +23526,7 @@
         <x:v>https://homepage.hit.edu.cn/wangxiuhong</x:v>
       </x:c>
       <x:c r="F102" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G102" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/wangxiuhong</x:v>
@@ -23535,7 +23535,7 @@
         <x:v>https://homepage.hit.edu.cn/wangxiuhong</x:v>
       </x:c>
       <x:c r="I102" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J102" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -23562,7 +23562,7 @@
         <x:v>https://homepage.hit.edu.cn/wangxiuhong</x:v>
       </x:c>
       <x:c r="F103" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G103" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/wangxiuhong</x:v>
@@ -23571,7 +23571,7 @@
         <x:v>https://homepage.hit.edu.cn/wangxiuhong</x:v>
       </x:c>
       <x:c r="I103" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J103" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -23598,7 +23598,7 @@
         <x:v>https://homepage.hit.edu.cn/yanxiaozhen</x:v>
       </x:c>
       <x:c r="F104" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G104" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/yanxiaozhen</x:v>
@@ -23607,7 +23607,7 @@
         <x:v>https://homepage.hit.edu.cn/yanxiaozhen</x:v>
       </x:c>
       <x:c r="I104" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J104" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -23634,7 +23634,7 @@
         <x:v>https://homepage.hit.edu.cn/yanxiaozhen</x:v>
       </x:c>
       <x:c r="F105" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G105" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/yanxiaozhen</x:v>
@@ -23643,7 +23643,7 @@
         <x:v>https://homepage.hit.edu.cn/yanxiaozhen</x:v>
       </x:c>
       <x:c r="I105" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J105" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -23672,7 +23672,7 @@
         <x:v>https://doi.org/10.12179/1672-4550.20180452</x:v>
       </x:c>
       <x:c r="F106" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G106" s="6" t="str">
         <x:v>https://www.sy.uestc.edu.cn/cn/article/pdf/preview/10.12179/1672-4550.20180452.pdf</x:v>
@@ -23681,7 +23681,7 @@
         <x:v>https://homepage.hit.edu.cn/yanxiaozhen</x:v>
       </x:c>
       <x:c r="I106" s="6" t="str">
-        <x:v>article_metadata_verified</x:v>
+        <x:v>文章书目元数据已核；不等于全部成果或全文发布。；article_metadata_verified</x:v>
       </x:c>
       <x:c r="J106" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：文章书目元数据已核；不等于全部成果或全文发布。</x:v>
@@ -23708,7 +23708,7 @@
         <x:v>https://homepage.hit.edu.cn/zhaowanlong</x:v>
       </x:c>
       <x:c r="F107" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G107" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/zhaowanlong</x:v>
@@ -23717,7 +23717,7 @@
         <x:v>https://homepage.hit.edu.cn/zhaowanlong</x:v>
       </x:c>
       <x:c r="I107" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J107" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -23744,7 +23744,7 @@
         <x:v>https://homepage.hit.edu.cn/zhaowanlong</x:v>
       </x:c>
       <x:c r="F108" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G108" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/zhaowanlong</x:v>
@@ -23753,7 +23753,7 @@
         <x:v>https://homepage.hit.edu.cn/zhaowanlong</x:v>
       </x:c>
       <x:c r="I108" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J108" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -23780,7 +23780,7 @@
         <x:v>https://homepage.hit.edu.cn/zhaowanlong</x:v>
       </x:c>
       <x:c r="F109" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G109" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/zhaowanlong</x:v>
@@ -23789,7 +23789,7 @@
         <x:v>https://homepage.hit.edu.cn/zhaowanlong</x:v>
       </x:c>
       <x:c r="I109" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J109" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -23814,7 +23814,7 @@
       <x:c r="D110" s="6" t="str"/>
       <x:c r="E110" s="6" t="str"/>
       <x:c r="F110" s="6" t="str">
-        <x:v>conference_paper</x:v>
+        <x:v>会议论文；conference_paper</x:v>
       </x:c>
       <x:c r="G110" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/xuejinghong</x:v>
@@ -23823,7 +23823,7 @@
         <x:v>https://homepage.hit.edu.cn/xuejinghong</x:v>
       </x:c>
       <x:c r="I110" s="6" t="str">
-        <x:v>bibliography_only_no_verified_article_link</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；bibliography_only_no_verified_article_link</x:v>
       </x:c>
       <x:c r="J110" s="6" t="str">
         <x:v>本人书目列题名及会议年；作者顺序、页码、DOI及独立链接未核实。 成果类型：会议论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -23846,7 +23846,7 @@
       <x:c r="D111" s="6" t="str"/>
       <x:c r="E111" s="6" t="str"/>
       <x:c r="F111" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G111" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/xuejinghong</x:v>
@@ -23855,7 +23855,7 @@
         <x:v>https://homepage.hit.edu.cn/xuejinghong</x:v>
       </x:c>
       <x:c r="I111" s="6" t="str">
-        <x:v>bibliography_only_no_verified_article_link</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；bibliography_only_no_verified_article_link</x:v>
       </x:c>
       <x:c r="J111" s="6" t="str">
         <x:v>本人公开书目列题名和刊名；其他书目字段未披露。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -23878,7 +23878,7 @@
       <x:c r="D112" s="6" t="str"/>
       <x:c r="E112" s="6" t="str"/>
       <x:c r="F112" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G112" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/xuejinghong</x:v>
@@ -23887,7 +23887,7 @@
         <x:v>https://homepage.hit.edu.cn/xuejinghong</x:v>
       </x:c>
       <x:c r="I112" s="6" t="str">
-        <x:v>bibliography_only_no_verified_article_link</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；bibliography_only_no_verified_article_link</x:v>
       </x:c>
       <x:c r="J112" s="6" t="str">
         <x:v>本人公开书目列题名和刊名；其他书目字段未披露。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -23916,7 +23916,7 @@
         <x:v>https://arxiv.org/abs/2207.02541</x:v>
       </x:c>
       <x:c r="F113" s="6" t="str">
-        <x:v>conference_paper</x:v>
+        <x:v>会议论文；conference_paper</x:v>
       </x:c>
       <x:c r="G113" s="6" t="str">
         <x:v>https://arxiv.org/abs/2207.02541</x:v>
@@ -23925,7 +23925,7 @@
         <x:v>https://homepage.hit.edu.cn/yuhaiyan</x:v>
       </x:c>
       <x:c r="I113" s="6" t="str">
-        <x:v>individual_article_page_verified</x:v>
+        <x:v>独立文章页书目已核，不表示全文复制或完整成果库。；individual_article_page_verified</x:v>
       </x:c>
       <x:c r="J113" s="6" t="str">
         <x:v>DOI为作者预印本DOI，非会议出版商DOI；会议名称由arXiv及本人书目相互印证。 成果类型：会议论文。 链接核验范围：独立文章页书目已核，不表示全文复制或完整成果库。</x:v>
@@ -23950,7 +23950,7 @@
       <x:c r="D114" s="6" t="str"/>
       <x:c r="E114" s="6" t="str"/>
       <x:c r="F114" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G114" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/yuhaiyan</x:v>
@@ -23959,7 +23959,7 @@
         <x:v>https://homepage.hit.edu.cn/yuhaiyan</x:v>
       </x:c>
       <x:c r="I114" s="6" t="str">
-        <x:v>bibliography_only_no_verified_article_link</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；bibliography_only_no_verified_article_link</x:v>
       </x:c>
       <x:c r="J114" s="6" t="str">
         <x:v>本人主页书目，未独立核验出版商链接；共同作者不作师承证据。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -23984,7 +23984,7 @@
       <x:c r="D115" s="6" t="str"/>
       <x:c r="E115" s="6" t="str"/>
       <x:c r="F115" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G115" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/yuhaiyan</x:v>
@@ -23993,7 +23993,7 @@
         <x:v>https://homepage.hit.edu.cn/yuhaiyan</x:v>
       </x:c>
       <x:c r="I115" s="6" t="str">
-        <x:v>bibliography_only_no_verified_article_link</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；bibliography_only_no_verified_article_link</x:v>
       </x:c>
       <x:c r="J115" s="6" t="str">
         <x:v>本人主页书目，未独立核验出版商链接。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -24018,7 +24018,7 @@
       <x:c r="D116" s="6" t="str"/>
       <x:c r="E116" s="6" t="str"/>
       <x:c r="F116" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G116" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/louyi</x:v>
@@ -24027,7 +24027,7 @@
         <x:v>https://homepage.hit.edu.cn/louyi</x:v>
       </x:c>
       <x:c r="I116" s="6" t="str">
-        <x:v>bibliography_only_no_verified_article_link</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；bibliography_only_no_verified_article_link</x:v>
       </x:c>
       <x:c r="J116" s="6" t="str">
         <x:v>本人书目列2026-01；卷页及DOI未核实。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -24052,7 +24052,7 @@
       <x:c r="D117" s="6" t="str"/>
       <x:c r="E117" s="6" t="str"/>
       <x:c r="F117" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G117" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/louyi</x:v>
@@ -24061,7 +24061,7 @@
         <x:v>https://homepage.hit.edu.cn/louyi</x:v>
       </x:c>
       <x:c r="I117" s="6" t="str">
-        <x:v>bibliography_only_no_verified_article_link</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；bibliography_only_no_verified_article_link</x:v>
       </x:c>
       <x:c r="J117" s="6" t="str">
         <x:v>本人书目列2025-03；出版商链接读取遇429，未重试或以绕行方式访问；卷页与DOI未纳入未验证字段。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -24086,7 +24086,7 @@
       <x:c r="D118" s="6" t="str"/>
       <x:c r="E118" s="6" t="str"/>
       <x:c r="F118" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G118" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/louyi</x:v>
@@ -24095,7 +24095,7 @@
         <x:v>https://homepage.hit.edu.cn/louyi</x:v>
       </x:c>
       <x:c r="I118" s="6" t="str">
-        <x:v>bibliography_only_no_verified_article_link</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；bibliography_only_no_verified_article_link</x:v>
       </x:c>
       <x:c r="J118" s="6" t="str">
         <x:v>本人书目列2024-11；独立出版商链接未核实。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -24120,7 +24120,7 @@
       <x:c r="D119" s="6" t="str"/>
       <x:c r="E119" s="6" t="str"/>
       <x:c r="F119" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G119" s="6" t="str">
         <x:v>https://wave-opt.lab.uic.edu/journal-papers/</x:v>
@@ -24129,7 +24129,7 @@
         <x:v>https://homepage.hit.edu.cn/fengxiang</x:v>
       </x:c>
       <x:c r="I119" s="6" t="str">
-        <x:v>bibliography_only_no_verified_article_link</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；bibliography_only_no_verified_article_link</x:v>
       </x:c>
       <x:c r="J119" s="6" t="str">
         <x:v>本人主页同题书目归属确认；UIC官方书目补全作者和页码。未把DOI搜索线索当已验证字段。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -24154,7 +24154,7 @@
       <x:c r="D120" s="6" t="str"/>
       <x:c r="E120" s="6" t="str"/>
       <x:c r="F120" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G120" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/fengxiang</x:v>
@@ -24163,7 +24163,7 @@
         <x:v>https://homepage.hit.edu.cn/fengxiang</x:v>
       </x:c>
       <x:c r="I120" s="6" t="str">
-        <x:v>bibliography_only_no_verified_article_link</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；bibliography_only_no_verified_article_link</x:v>
       </x:c>
       <x:c r="J120" s="6" t="str">
         <x:v>按本人书目记录；独立出版商元数据未核验。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -24188,7 +24188,7 @@
       <x:c r="D121" s="6" t="str"/>
       <x:c r="E121" s="6" t="str"/>
       <x:c r="F121" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G121" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/fengxiang</x:v>
@@ -24197,7 +24197,7 @@
         <x:v>https://homepage.hit.edu.cn/fengxiang</x:v>
       </x:c>
       <x:c r="I121" s="6" t="str">
-        <x:v>bibliography_only_no_verified_article_link</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；bibliography_only_no_verified_article_link</x:v>
       </x:c>
       <x:c r="J121" s="6" t="str">
         <x:v>本人书目作者为“Zhao Z S, Feng X, Lin Y, et al.”，所列仅已披露作者，非完整作者表。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -24226,7 +24226,7 @@
         <x:v>https://doi.org/10.1063/5.0287957</x:v>
       </x:c>
       <x:c r="F122" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G122" s="6" t="str">
         <x:v>https://doi.org/10.1063/5.0287957</x:v>
@@ -24235,7 +24235,7 @@
         <x:v>https://homepage.hit.edu.cn/tangshuai</x:v>
       </x:c>
       <x:c r="I122" s="6" t="str">
-        <x:v>individual_article_page_verified</x:v>
+        <x:v>独立文章页书目已核，不表示全文复制或完整成果库。；individual_article_page_verified</x:v>
       </x:c>
       <x:c r="J122" s="6" t="str">
         <x:v>出版商列唐帅为威海信息学院，ORCID与2023论文相同；本文只取公开书目。 成果类型：期刊论文。 链接核验范围：独立文章页书目已核，不表示全文复制或完整成果库。</x:v>
@@ -24264,7 +24264,7 @@
         <x:v>https://pubs.aip.org/aip/apl/article-abstract/122/21/212201/2892528/Unidirectional-beam-splitting-in-acoustic?redirectedFrom=fulltext</x:v>
       </x:c>
       <x:c r="F123" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G123" s="6" t="str">
         <x:v>https://pubs.aip.org/aip/apl/article-abstract/122/21/212201/2892528/Unidirectional-beam-splitting-in-acoustic?redirectedFrom=fulltext</x:v>
@@ -24273,7 +24273,7 @@
         <x:v>https://homepage.hit.edu.cn/tangshuai</x:v>
       </x:c>
       <x:c r="I123" s="6" t="str">
-        <x:v>indexed_article_link_not_live_verified</x:v>
+        <x:v>仅索引书目与链接，文章落地页未直接核实。；indexed_article_link_not_live_verified</x:v>
       </x:c>
       <x:c r="J123" s="6" t="str">
         <x:v>出版商搜索索引完整元数据与姜永远官方书目相符；直开Cache miss，链接保守标未实时验证。 成果类型：期刊论文。 链接核验范围：仅索引书目与链接，文章落地页未直接核实。</x:v>
@@ -24300,7 +24300,7 @@
         <x:v>https://homepage.hit.edu.cn/LIYANG13836167631</x:v>
       </x:c>
       <x:c r="F124" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G124" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/LIYANG13836167631</x:v>
@@ -24309,7 +24309,7 @@
         <x:v>https://homepage.hit.edu.cn/LIYANG13836167631</x:v>
       </x:c>
       <x:c r="I124" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J124" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -24336,7 +24336,7 @@
         <x:v>https://homepage.hit.edu.cn/LIYANG13836167631</x:v>
       </x:c>
       <x:c r="F125" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G125" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/LIYANG13836167631</x:v>
@@ -24345,7 +24345,7 @@
         <x:v>https://homepage.hit.edu.cn/LIYANG13836167631</x:v>
       </x:c>
       <x:c r="I125" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J125" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -24372,7 +24372,7 @@
         <x:v>https://homepage.hit.edu.cn/LIYANG13836167631</x:v>
       </x:c>
       <x:c r="F126" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G126" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/LIYANG13836167631</x:v>
@@ -24381,7 +24381,7 @@
         <x:v>https://homepage.hit.edu.cn/LIYANG13836167631</x:v>
       </x:c>
       <x:c r="I126" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J126" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -24408,7 +24408,7 @@
         <x:v>https://homepage.hit.edu.cn/zhouhongjuan</x:v>
       </x:c>
       <x:c r="F127" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G127" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/zhouhongjuan</x:v>
@@ -24417,7 +24417,7 @@
         <x:v>https://homepage.hit.edu.cn/zhouhongjuan</x:v>
       </x:c>
       <x:c r="I127" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J127" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -24444,7 +24444,7 @@
         <x:v>https://homepage.hit.edu.cn/zhouhongjuan</x:v>
       </x:c>
       <x:c r="F128" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G128" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/zhouhongjuan</x:v>
@@ -24453,7 +24453,7 @@
         <x:v>https://homepage.hit.edu.cn/zhouhongjuan</x:v>
       </x:c>
       <x:c r="I128" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J128" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -24480,7 +24480,7 @@
         <x:v>https://homepage.hit.edu.cn/zhouhongjuan</x:v>
       </x:c>
       <x:c r="F129" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G129" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/zhouhongjuan</x:v>
@@ -24489,7 +24489,7 @@
         <x:v>https://homepage.hit.edu.cn/zhouhongjuan</x:v>
       </x:c>
       <x:c r="I129" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J129" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -24518,7 +24518,7 @@
         <x:v>https://doi.org/10.3390/s22176474</x:v>
       </x:c>
       <x:c r="F130" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G130" s="6" t="str">
         <x:v>https://pubmed.ncbi.nlm.nih.gov/36080932/</x:v>
@@ -24527,7 +24527,7 @@
         <x:v>https://homepage.hit.edu.cn/liyingchun</x:v>
       </x:c>
       <x:c r="I130" s="6" t="str">
-        <x:v>article_metadata_verified</x:v>
+        <x:v>文章书目元数据已核；不等于全部成果或全文发布。；article_metadata_verified</x:v>
       </x:c>
       <x:c r="J130" s="6" t="str">
         <x:v>PubMed实际读取署名与威海学院单位；出版者MDPI直连429后未重试，只用独立公开题录，不读取全文。 成果类型：期刊论文。 链接核验范围：文章书目元数据已核；不等于全部成果或全文发布。</x:v>
@@ -24554,7 +24554,7 @@
         <x:v>https://homepage.hit.edu.cn/caobingxia</x:v>
       </x:c>
       <x:c r="F131" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G131" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/caobingxia</x:v>
@@ -24563,7 +24563,7 @@
         <x:v>https://homepage.hit.edu.cn/caobingxia</x:v>
       </x:c>
       <x:c r="I131" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J131" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -24590,7 +24590,7 @@
         <x:v>https://homepage.hit.edu.cn/caobingxia</x:v>
       </x:c>
       <x:c r="F132" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G132" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/caobingxia</x:v>
@@ -24599,7 +24599,7 @@
         <x:v>https://homepage.hit.edu.cn/caobingxia</x:v>
       </x:c>
       <x:c r="I132" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J132" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -24626,7 +24626,7 @@
         <x:v>https://homepage.hit.edu.cn/caobingxia</x:v>
       </x:c>
       <x:c r="F133" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G133" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/caobingxia</x:v>
@@ -24635,7 +24635,7 @@
         <x:v>https://homepage.hit.edu.cn/caobingxia</x:v>
       </x:c>
       <x:c r="I133" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J133" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -24662,7 +24662,7 @@
         <x:v>https://homepage.hit.edu.cn/MaYiming</x:v>
       </x:c>
       <x:c r="F134" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G134" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/MaYiming</x:v>
@@ -24671,7 +24671,7 @@
         <x:v>https://homepage.hit.edu.cn/MaYiming</x:v>
       </x:c>
       <x:c r="I134" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J134" s="6" t="str">
         <x:v>书目字段来自本人官方论文清单，未将主页链接标为单篇论文链接。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -24698,7 +24698,7 @@
         <x:v>https://homepage.hit.edu.cn/MaYiming</x:v>
       </x:c>
       <x:c r="F135" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G135" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/MaYiming</x:v>
@@ -24707,7 +24707,7 @@
         <x:v>https://homepage.hit.edu.cn/MaYiming</x:v>
       </x:c>
       <x:c r="I135" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J135" s="6" t="str">
         <x:v>书目字段来自本人官方论文清单，未将主页链接标为单篇论文链接。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -24734,7 +24734,7 @@
         <x:v>https://homepage.hit.edu.cn/MaYiming</x:v>
       </x:c>
       <x:c r="F136" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G136" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/MaYiming</x:v>
@@ -24743,7 +24743,7 @@
         <x:v>https://homepage.hit.edu.cn/MaYiming</x:v>
       </x:c>
       <x:c r="I136" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J136" s="6" t="str">
         <x:v>书目字段来自本人官方论文清单，未将主页链接标为单篇论文链接。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -24770,7 +24770,7 @@
         <x:v>https://homepage.hit.edu.cn/kuangjiyuan</x:v>
       </x:c>
       <x:c r="F137" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G137" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/kuangjiyuan</x:v>
@@ -24779,7 +24779,7 @@
         <x:v>https://homepage.hit.edu.cn/kuangjiyuan</x:v>
       </x:c>
       <x:c r="I137" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J137" s="6" t="str">
         <x:v>书目字段来自本人官方论文清单，未将主页链接标为单篇论文链接。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -24806,7 +24806,7 @@
         <x:v>https://homepage.hit.edu.cn/kuangjiyuan</x:v>
       </x:c>
       <x:c r="F138" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G138" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/kuangjiyuan</x:v>
@@ -24815,7 +24815,7 @@
         <x:v>https://homepage.hit.edu.cn/kuangjiyuan</x:v>
       </x:c>
       <x:c r="I138" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J138" s="6" t="str">
         <x:v>书目字段来自本人官方论文清单，未将主页链接标为单篇论文链接。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -24842,7 +24842,7 @@
         <x:v>https://homepage.hit.edu.cn/kuangjiyuan</x:v>
       </x:c>
       <x:c r="F139" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G139" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/kuangjiyuan</x:v>
@@ -24851,7 +24851,7 @@
         <x:v>https://homepage.hit.edu.cn/kuangjiyuan</x:v>
       </x:c>
       <x:c r="I139" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J139" s="6" t="str">
         <x:v>书目字段来自本人官方论文清单，未将主页链接标为单篇论文链接。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -24878,7 +24878,7 @@
         <x:v>https://homepage.hit.edu.cn/linxinpo</x:v>
       </x:c>
       <x:c r="F140" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G140" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/linxinpo</x:v>
@@ -24887,7 +24887,7 @@
         <x:v>https://homepage.hit.edu.cn/linxinpo</x:v>
       </x:c>
       <x:c r="I140" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J140" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -24914,7 +24914,7 @@
         <x:v>https://homepage.hit.edu.cn/linxinpo</x:v>
       </x:c>
       <x:c r="F141" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G141" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/linxinpo</x:v>
@@ -24923,7 +24923,7 @@
         <x:v>https://homepage.hit.edu.cn/linxinpo</x:v>
       </x:c>
       <x:c r="I141" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J141" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -24950,7 +24950,7 @@
         <x:v>https://homepage.hit.edu.cn/linxinpo</x:v>
       </x:c>
       <x:c r="F142" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G142" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/linxinpo</x:v>
@@ -24959,7 +24959,7 @@
         <x:v>https://homepage.hit.edu.cn/linxinpo</x:v>
       </x:c>
       <x:c r="I142" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J142" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -24986,7 +24986,7 @@
         <x:v>https://homepage.hit.edu.cn/jiaguangle</x:v>
       </x:c>
       <x:c r="F143" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G143" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/jiaguangle</x:v>
@@ -24995,7 +24995,7 @@
         <x:v>https://homepage.hit.edu.cn/jiaguangle</x:v>
       </x:c>
       <x:c r="I143" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J143" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -25022,7 +25022,7 @@
         <x:v>https://homepage.hit.edu.cn/jiaguangle</x:v>
       </x:c>
       <x:c r="F144" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G144" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/jiaguangle</x:v>
@@ -25031,7 +25031,7 @@
         <x:v>https://homepage.hit.edu.cn/jiaguangle</x:v>
       </x:c>
       <x:c r="I144" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J144" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -25058,7 +25058,7 @@
         <x:v>https://homepage.hit.edu.cn/jiaguangle</x:v>
       </x:c>
       <x:c r="F145" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G145" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/jiaguangle</x:v>
@@ -25067,7 +25067,7 @@
         <x:v>https://homepage.hit.edu.cn/jiaguangle</x:v>
       </x:c>
       <x:c r="I145" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J145" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -25092,7 +25092,7 @@
         <x:v>https://homepage.hit.edu.cn/shaoshuai</x:v>
       </x:c>
       <x:c r="F146" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G146" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/shaoshuai</x:v>
@@ -25101,7 +25101,7 @@
         <x:v>https://homepage.hit.edu.cn/shaoshuai</x:v>
       </x:c>
       <x:c r="I146" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J146" s="6" t="str">
         <x:v>官网成果栏目未列年份、DOI和逐篇链接，不猜。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -25126,7 +25126,7 @@
         <x:v>https://homepage.hit.edu.cn/shaoshuai</x:v>
       </x:c>
       <x:c r="F147" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G147" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/shaoshuai</x:v>
@@ -25135,7 +25135,7 @@
         <x:v>https://homepage.hit.edu.cn/shaoshuai</x:v>
       </x:c>
       <x:c r="I147" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J147" s="6" t="str">
         <x:v>官网成果栏目未列年份、DOI和逐篇链接，不猜。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -25162,7 +25162,7 @@
         <x:v>https://homepage.hit.edu.cn/sunyongjin</x:v>
       </x:c>
       <x:c r="F148" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G148" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/sunyongjin</x:v>
@@ -25171,7 +25171,7 @@
         <x:v>https://homepage.hit.edu.cn/sunyongjin</x:v>
       </x:c>
       <x:c r="I148" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J148" s="6" t="str">
         <x:v>本人官网代表作第1项；仅修复标题中Improvingthe、decompositionmethod的连写空格。主页不是单篇论文链接，DOI未提供。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -25198,7 +25198,7 @@
         <x:v>https://homepage.hit.edu.cn/sunyongjin</x:v>
       </x:c>
       <x:c r="F149" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G149" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/sunyongjin</x:v>
@@ -25207,7 +25207,7 @@
         <x:v>https://homepage.hit.edu.cn/sunyongjin</x:v>
       </x:c>
       <x:c r="I149" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J149" s="6" t="str">
         <x:v>本人官网代表作第2项；只修复SeafloorTopography与OptimizationMethod连写空格，不改写标题措辞。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -25234,7 +25234,7 @@
         <x:v>https://homepage.hit.edu.cn/sunyongjin</x:v>
       </x:c>
       <x:c r="F150" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G150" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/sunyongjin</x:v>
@@ -25243,7 +25243,7 @@
         <x:v>https://homepage.hit.edu.cn/sunyongjin</x:v>
       </x:c>
       <x:c r="I150" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J150" s="6" t="str">
         <x:v>本人官网代表作第3项；只修复Accuracyof、CombinedModification连写空格。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -25270,7 +25270,7 @@
         <x:v>https://homepage.hit.edu.cn/mengxiangtian</x:v>
       </x:c>
       <x:c r="F151" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G151" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/mengxiangtian</x:v>
@@ -25279,7 +25279,7 @@
         <x:v>https://homepage.hit.edu.cn/mengxiangtian</x:v>
       </x:c>
       <x:c r="I151" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J151" s="6" t="str">
         <x:v>本人官网代表性论文第1项；原文et al.，仅列具名作者，不冒充完整作者清单。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -25306,7 +25306,7 @@
         <x:v>https://homepage.hit.edu.cn/mengxiangtian</x:v>
       </x:c>
       <x:c r="F152" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G152" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/mengxiangtian</x:v>
@@ -25315,7 +25315,7 @@
         <x:v>https://homepage.hit.edu.cn/mengxiangtian</x:v>
       </x:c>
       <x:c r="I152" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J152" s="6" t="str">
         <x:v>本人官网代表性论文第2项；原文et al.，仅列具名作者。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -25342,7 +25342,7 @@
         <x:v>https://homepage.hit.edu.cn/mengxiangtian</x:v>
       </x:c>
       <x:c r="F153" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G153" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/mengxiangtian</x:v>
@@ -25351,7 +25351,7 @@
         <x:v>https://homepage.hit.edu.cn/mengxiangtian</x:v>
       </x:c>
       <x:c r="I153" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J153" s="6" t="str">
         <x:v>本人官网代表性论文第3项；原文et al.，仅列具名作者；不将星号作者标记作为师承证据。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -25378,7 +25378,7 @@
         <x:v>https://homepage.hit.edu.cn/liuxiaoning</x:v>
       </x:c>
       <x:c r="F154" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G154" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/liuxiaoning</x:v>
@@ -25387,7 +25387,7 @@
         <x:v>https://homepage.hit.edu.cn/liuxiaoning</x:v>
       </x:c>
       <x:c r="I154" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J154" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -25414,7 +25414,7 @@
         <x:v>https://homepage.hit.edu.cn/liuxiaoning</x:v>
       </x:c>
       <x:c r="F155" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G155" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/liuxiaoning</x:v>
@@ -25423,7 +25423,7 @@
         <x:v>https://homepage.hit.edu.cn/liuxiaoning</x:v>
       </x:c>
       <x:c r="I155" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J155" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -25450,7 +25450,7 @@
         <x:v>https://homepage.hit.edu.cn/liuxiaoning</x:v>
       </x:c>
       <x:c r="F156" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G156" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/liuxiaoning</x:v>
@@ -25459,7 +25459,7 @@
         <x:v>https://homepage.hit.edu.cn/liuxiaoning</x:v>
       </x:c>
       <x:c r="I156" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J156" s="6" t="str">
         <x:v>成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -25486,7 +25486,7 @@
         <x:v>https://homepage.hit.edu.cn/HanYong?lang=zh</x:v>
       </x:c>
       <x:c r="F157" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G157" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/HanYong?lang=zh</x:v>
@@ -25495,7 +25495,7 @@
         <x:v>https://homepage.hit.edu.cn/HanYong?lang=zh</x:v>
       </x:c>
       <x:c r="I157" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J157" s="6" t="str">
         <x:v>本人官方论文清单的精选书目；原文作者含et al./等，所列为已显示作者而非完整作者表；主页链接不是单篇文章链接。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -25522,7 +25522,7 @@
         <x:v>https://homepage.hit.edu.cn/HanYong?lang=zh</x:v>
       </x:c>
       <x:c r="F158" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G158" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/HanYong?lang=zh</x:v>
@@ -25531,7 +25531,7 @@
         <x:v>https://homepage.hit.edu.cn/HanYong?lang=zh</x:v>
       </x:c>
       <x:c r="I158" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J158" s="6" t="str">
         <x:v>本人官方论文清单的精选书目；原文作者含et al./等，所列为已显示作者而非完整作者表；主页链接不是单篇文章链接。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -25558,7 +25558,7 @@
         <x:v>https://homepage.hit.edu.cn/HanYong?lang=zh</x:v>
       </x:c>
       <x:c r="F159" s="6" t="str">
-        <x:v>journal_article</x:v>
+        <x:v>期刊论文；journal_article</x:v>
       </x:c>
       <x:c r="G159" s="6" t="str">
         <x:v>https://homepage.hit.edu.cn/HanYong?lang=zh</x:v>
@@ -25567,7 +25567,7 @@
         <x:v>https://homepage.hit.edu.cn/HanYong?lang=zh</x:v>
       </x:c>
       <x:c r="I159" s="6" t="str">
-        <x:v>official_publication_list_only</x:v>
+        <x:v>仅本人官网精选书目，独立文章页未核。；official_publication_list_only</x:v>
       </x:c>
       <x:c r="J159" s="6" t="str">
         <x:v>本人官方论文清单的精选书目；原文作者含et al./等，所列为已显示作者而非完整作者表；主页链接不是单篇文章链接。 成果类型：期刊论文。 链接核验范围：仅本人官网精选书目，独立文章页未核。</x:v>
@@ -25582,7 +25582,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc2b4f673d164a27"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ed2a5ed192e47e4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31330,7 +31330,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d19966c8f3542e2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd19462186e144da"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>